<commit_message>
docs: close Phase 0 (item 0.4 merged), update progress and Gantt
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014MvxPtyCrWLViJ8svf2cG9
</commit_message>
<xml_diff>
--- a/reports/gantt.xlsx
+++ b/reports/gantt.xlsx
@@ -562,7 +562,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Inicio 2026-10-11 · Fin 2027-03-12 · generado 2026-10-11 desde PLAN.md</t>
+          <t>Inicio 2026-10-11 · Fin 2027-03-12 · generado 2026-10-12 desde PLAN.md</t>
         </is>
       </c>
     </row>
@@ -774,14 +774,16 @@
         <v>46307</v>
       </c>
       <c r="F6" s="11" t="n"/>
-      <c r="G6" s="11" t="n"/>
+      <c r="G6" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I6" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" s="10">
         <f>IF(AND(G6&lt;&gt;"",E6&lt;&gt;""),G6-E6,"")</f>
@@ -832,14 +834,16 @@
         <v>46309</v>
       </c>
       <c r="F7" s="11" t="n"/>
-      <c r="G7" s="11" t="n"/>
+      <c r="G7" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" s="10">
         <f>IF(AND(G7&lt;&gt;"",E7&lt;&gt;""),G7-E7,"")</f>
@@ -890,14 +894,16 @@
         <v>46310</v>
       </c>
       <c r="F8" s="11" t="n"/>
-      <c r="G8" s="11" t="n"/>
+      <c r="G8" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" s="10">
         <f>IF(AND(G8&lt;&gt;"",E8&lt;&gt;""),G8-E8,"")</f>
@@ -951,11 +957,11 @@
       <c r="G9" s="11" t="n"/>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I9" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" s="10">
         <f>IF(AND(G9&lt;&gt;"",E9&lt;&gt;""),G9-E9,"")</f>

</xml_diff>

<commit_message>
docs: regenerate Gantt after items 1.1-1.6
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014MvxPtyCrWLViJ8svf2cG9
</commit_message>
<xml_diff>
--- a/reports/gantt.xlsx
+++ b/reports/gantt.xlsx
@@ -954,7 +954,9 @@
         <v>46311</v>
       </c>
       <c r="F9" s="11" t="n"/>
-      <c r="G9" s="11" t="n"/>
+      <c r="G9" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
           <t>Completado</t>
@@ -1078,14 +1080,16 @@
         <v>46315</v>
       </c>
       <c r="F11" s="11" t="n"/>
-      <c r="G11" s="11" t="n"/>
+      <c r="G11" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11" s="10">
         <f>IF(AND(G11&lt;&gt;"",E11&lt;&gt;""),G11-E11,"")</f>
@@ -1136,14 +1140,16 @@
         <v>46321</v>
       </c>
       <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
+      <c r="G12" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I12" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" s="10">
         <f>IF(AND(G12&lt;&gt;"",E12&lt;&gt;""),G12-E12,"")</f>
@@ -1194,14 +1200,16 @@
         <v>46328</v>
       </c>
       <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
+      <c r="G13" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I13" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" s="10">
         <f>IF(AND(G13&lt;&gt;"",E13&lt;&gt;""),G13-E13,"")</f>
@@ -1252,14 +1260,16 @@
         <v>46334</v>
       </c>
       <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n"/>
+      <c r="G14" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H14" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I14" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" s="10">
         <f>IF(AND(G14&lt;&gt;"",E14&lt;&gt;""),G14-E14,"")</f>
@@ -1310,14 +1320,16 @@
         <v>46337</v>
       </c>
       <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
+      <c r="G15" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I15" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15" s="10">
         <f>IF(AND(G15&lt;&gt;"",E15&lt;&gt;""),G15-E15,"")</f>
@@ -1368,14 +1380,16 @@
         <v>46341</v>
       </c>
       <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n"/>
+      <c r="G16" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H16" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I16" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" s="10">
         <f>IF(AND(G16&lt;&gt;"",E16&lt;&gt;""),G16-E16,"")</f>

</xml_diff>

<commit_message>
feat(tracking): change means of transport mid-session (item 2.9)
- Active session: "Medio: … · cambiar" opens a transport dialog; the
  segment stores the new transport and sampling profile, a
  TRANSPORT_CHANGE text note records time and position, and the running
  service retunes the GPS request and point filter without closing the
  stage (filter re-seeded with the last accepted fix, battery saver kept)
- Timeline event TransportChange rendered in the trip detail
- gpx-replay: --skip to continue a replay
- Evidence: docs/notes/evidencia/fase-2/2.9-cambio-de-medio.md; Gantt
  regenerated

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014MvxPtyCrWLViJ8svf2cG9
</commit_message>
<xml_diff>
--- a/reports/gantt.xlsx
+++ b/reports/gantt.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG55"/>
+  <dimension ref="A1:AG56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1137,7 +1137,7 @@
         <v>46315</v>
       </c>
       <c r="E12" s="11" t="n">
-        <v>46321</v>
+        <v>46320</v>
       </c>
       <c r="F12" s="11" t="n"/>
       <c r="G12" s="11" t="n">
@@ -1194,10 +1194,10 @@
         <v>3</v>
       </c>
       <c r="D13" s="11" t="n">
-        <v>46321</v>
+        <v>46320</v>
       </c>
       <c r="E13" s="11" t="n">
-        <v>46328</v>
+        <v>46327</v>
       </c>
       <c r="F13" s="11" t="n"/>
       <c r="G13" s="11" t="n">
@@ -1254,10 +1254,10 @@
         <v>2.5</v>
       </c>
       <c r="D14" s="11" t="n">
-        <v>46328</v>
+        <v>46327</v>
       </c>
       <c r="E14" s="11" t="n">
-        <v>46334</v>
+        <v>46332</v>
       </c>
       <c r="F14" s="11" t="n"/>
       <c r="G14" s="11" t="n">
@@ -1314,10 +1314,10 @@
         <v>1.5</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>46334</v>
+        <v>46332</v>
       </c>
       <c r="E15" s="11" t="n">
-        <v>46337</v>
+        <v>46335</v>
       </c>
       <c r="F15" s="11" t="n"/>
       <c r="G15" s="11" t="n">
@@ -1374,10 +1374,10 @@
         <v>2</v>
       </c>
       <c r="D16" s="11" t="n">
-        <v>46337</v>
+        <v>46335</v>
       </c>
       <c r="E16" s="11" t="n">
-        <v>46341</v>
+        <v>46339</v>
       </c>
       <c r="F16" s="11" t="n"/>
       <c r="G16" s="11" t="n">
@@ -1434,10 +1434,10 @@
         <v>0.5</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>46341</v>
+        <v>46339</v>
       </c>
       <c r="E17" s="11" t="n">
-        <v>46342</v>
+        <v>46340</v>
       </c>
       <c r="F17" s="11" t="n"/>
       <c r="G17" s="11" t="n"/>
@@ -1489,22 +1489,22 @@
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>12</v>
+        <v>12.5</v>
       </c>
       <c r="D18" s="7">
-        <f>IF(COUNT(D19:D26)=0,"",MIN(D19:D26))</f>
+        <f>IF(COUNT(D19:D27)=0,"",MIN(D19:D27))</f>
         <v/>
       </c>
       <c r="E18" s="7">
-        <f>IF(COUNT(E19:E26)=0,"",MAX(E19:E26))</f>
+        <f>IF(COUNT(E19:E27)=0,"",MAX(E19:E27))</f>
         <v/>
       </c>
       <c r="F18" s="7">
-        <f>IF(COUNT(F19:F26)=0,"",MIN(F19:F26))</f>
+        <f>IF(COUNT(F19:F27)=0,"",MIN(F19:F27))</f>
         <v/>
       </c>
       <c r="G18" s="7">
-        <f>IF(COUNT(G19:G26)=0,"",MAX(G19:G26))</f>
+        <f>IF(COUNT(G19:G27)=0,"",MAX(G19:G27))</f>
         <v/>
       </c>
       <c r="H18" s="5">
@@ -1512,7 +1512,7 @@
         <v/>
       </c>
       <c r="I18" s="8">
-        <f>IF(COUNT(I19:I26)=0,"",AVERAGE(I19:I26))</f>
+        <f>IF(COUNT(I19:I27)=0,"",AVERAGE(I19:I27))</f>
         <v/>
       </c>
       <c r="J18" s="6">
@@ -1558,20 +1558,22 @@
         <v>1</v>
       </c>
       <c r="D19" s="11" t="n">
+        <v>46340</v>
+      </c>
+      <c r="E19" s="11" t="n">
         <v>46342</v>
       </c>
-      <c r="E19" s="11" t="n">
-        <v>46344</v>
-      </c>
       <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="G19" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I19" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" s="10">
         <f>IF(AND(G19&lt;&gt;"",E19&lt;&gt;""),G19-E19,"")</f>
@@ -1616,20 +1618,22 @@
         <v>2</v>
       </c>
       <c r="D20" s="11" t="n">
-        <v>46344</v>
+        <v>46342</v>
       </c>
       <c r="E20" s="11" t="n">
-        <v>46348</v>
+        <v>46346</v>
       </c>
       <c r="F20" s="11" t="n"/>
-      <c r="G20" s="11" t="n"/>
+      <c r="G20" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I20" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20" s="10">
         <f>IF(AND(G20&lt;&gt;"",E20&lt;&gt;""),G20-E20,"")</f>
@@ -1674,20 +1678,22 @@
         <v>1.5</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>46348</v>
+        <v>46346</v>
       </c>
       <c r="E21" s="11" t="n">
-        <v>46351</v>
+        <v>46349</v>
       </c>
       <c r="F21" s="11" t="n"/>
-      <c r="G21" s="11" t="n"/>
+      <c r="G21" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H21" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I21" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21" s="10">
         <f>IF(AND(G21&lt;&gt;"",E21&lt;&gt;""),G21-E21,"")</f>
@@ -1732,10 +1738,10 @@
         <v>2.5</v>
       </c>
       <c r="D22" s="11" t="n">
-        <v>46351</v>
+        <v>46349</v>
       </c>
       <c r="E22" s="11" t="n">
-        <v>46357</v>
+        <v>46354</v>
       </c>
       <c r="F22" s="11" t="n"/>
       <c r="G22" s="11" t="n"/>
@@ -1790,20 +1796,22 @@
         <v>0.5</v>
       </c>
       <c r="D23" s="11" t="n">
-        <v>46357</v>
+        <v>46354</v>
       </c>
       <c r="E23" s="11" t="n">
-        <v>46358</v>
+        <v>46355</v>
       </c>
       <c r="F23" s="11" t="n"/>
-      <c r="G23" s="11" t="n"/>
+      <c r="G23" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H23" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I23" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J23" s="10">
         <f>IF(AND(G23&lt;&gt;"",E23&lt;&gt;""),G23-E23,"")</f>
@@ -1848,20 +1856,22 @@
         <v>1.5</v>
       </c>
       <c r="D24" s="11" t="n">
+        <v>46355</v>
+      </c>
+      <c r="E24" s="11" t="n">
         <v>46358</v>
       </c>
-      <c r="E24" s="11" t="n">
-        <v>46361</v>
-      </c>
       <c r="F24" s="11" t="n"/>
-      <c r="G24" s="11" t="n"/>
+      <c r="G24" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H24" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I24" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" s="10">
         <f>IF(AND(G24&lt;&gt;"",E24&lt;&gt;""),G24-E24,"")</f>
@@ -1906,20 +1916,22 @@
         <v>2.5</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>46361</v>
+        <v>46358</v>
       </c>
       <c r="E25" s="11" t="n">
-        <v>46367</v>
+        <v>46363</v>
       </c>
       <c r="F25" s="11" t="n"/>
-      <c r="G25" s="11" t="n"/>
+      <c r="G25" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I25" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25" s="10">
         <f>IF(AND(G25&lt;&gt;"",E25&lt;&gt;""),G25-E25,"")</f>
@@ -1964,10 +1976,10 @@
         <v>0.5</v>
       </c>
       <c r="D26" s="11" t="n">
-        <v>46367</v>
+        <v>46363</v>
       </c>
       <c r="E26" s="11" t="n">
-        <v>46368</v>
+        <v>46364</v>
       </c>
       <c r="F26" s="11" t="n"/>
       <c r="G26" s="11" t="n"/>
@@ -2008,148 +2020,148 @@
       <c r="AG26" s="9" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>2.9</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Cambiar el medio de transporte durante la sesión (agregado 2026-10-12 a pedido del usuario): botón en la se...</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D27" s="11" t="n">
+        <v>46364</v>
+      </c>
+      <c r="E27" s="11" t="n">
+        <v>46365</v>
+      </c>
+      <c r="F27" s="11" t="n"/>
+      <c r="G27" s="11" t="n"/>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>Completado</t>
+        </is>
+      </c>
+      <c r="I27" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J27" s="10">
+        <f>IF(AND(G27&lt;&gt;"",E27&lt;&gt;""),G27-E27,"")</f>
+        <v/>
+      </c>
+      <c r="K27" s="9" t="n"/>
+      <c r="L27" s="9" t="n"/>
+      <c r="M27" s="9" t="n"/>
+      <c r="N27" s="9" t="n"/>
+      <c r="O27" s="9" t="n"/>
+      <c r="P27" s="9" t="n"/>
+      <c r="Q27" s="9" t="n"/>
+      <c r="R27" s="9" t="n"/>
+      <c r="S27" s="9" t="n"/>
+      <c r="T27" s="9" t="n"/>
+      <c r="U27" s="9" t="n"/>
+      <c r="V27" s="9" t="n"/>
+      <c r="W27" s="9" t="n"/>
+      <c r="X27" s="9" t="n"/>
+      <c r="Y27" s="9" t="n"/>
+      <c r="Z27" s="9" t="n"/>
+      <c r="AA27" s="9" t="n"/>
+      <c r="AB27" s="9" t="n"/>
+      <c r="AC27" s="9" t="n"/>
+      <c r="AD27" s="9" t="n"/>
+      <c r="AE27" s="9" t="n"/>
+      <c r="AF27" s="9" t="n"/>
+      <c r="AG27" s="9" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>F3</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>Fase 3 — Exportación, transcripción local y tareas largas</t>
         </is>
       </c>
-      <c r="C27" s="6" t="n">
+      <c r="C28" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="D27" s="7">
-        <f>IF(COUNT(D28:D34)=0,"",MIN(D28:D34))</f>
-        <v/>
-      </c>
-      <c r="E27" s="7">
-        <f>IF(COUNT(E28:E34)=0,"",MAX(E28:E34))</f>
-        <v/>
-      </c>
-      <c r="F27" s="7">
-        <f>IF(COUNT(F28:F34)=0,"",MIN(F28:F34))</f>
-        <v/>
-      </c>
-      <c r="G27" s="7">
-        <f>IF(COUNT(G28:G34)=0,"",MAX(G28:G34))</f>
-        <v/>
-      </c>
-      <c r="H27" s="5">
-        <f>IF(I27="","",IF(I27=1,"Completada",IF(I27=0,"Pendiente","En curso")))</f>
-        <v/>
-      </c>
-      <c r="I27" s="8">
-        <f>IF(COUNT(I28:I34)=0,"",AVERAGE(I28:I34))</f>
-        <v/>
-      </c>
-      <c r="J27" s="6">
-        <f>IF(AND(G27&lt;&gt;"",E27&lt;&gt;""),G27-E27,"")</f>
-        <v/>
-      </c>
-      <c r="K27" s="5" t="n"/>
-      <c r="L27" s="5" t="n"/>
-      <c r="M27" s="5" t="n"/>
-      <c r="N27" s="5" t="n"/>
-      <c r="O27" s="5" t="n"/>
-      <c r="P27" s="5" t="n"/>
-      <c r="Q27" s="5" t="n"/>
-      <c r="R27" s="5" t="n"/>
-      <c r="S27" s="5" t="n"/>
-      <c r="T27" s="5" t="n"/>
-      <c r="U27" s="5" t="n"/>
-      <c r="V27" s="5" t="n"/>
-      <c r="W27" s="5" t="n"/>
-      <c r="X27" s="5" t="n"/>
-      <c r="Y27" s="5" t="n"/>
-      <c r="Z27" s="5" t="n"/>
-      <c r="AA27" s="5" t="n"/>
-      <c r="AB27" s="5" t="n"/>
-      <c r="AC27" s="5" t="n"/>
-      <c r="AD27" s="5" t="n"/>
-      <c r="AE27" s="5" t="n"/>
-      <c r="AF27" s="5" t="n"/>
-      <c r="AG27" s="5" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
-        <is>
-          <t>3.1</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>`core/export`: `trip.json` + JSON Schema, GPX 1.1 con extensiones propias y de Garmin validado contra XSD,...</t>
-        </is>
-      </c>
-      <c r="C28" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="D28" s="11" t="n">
-        <v>46368</v>
-      </c>
-      <c r="E28" s="11" t="n">
-        <v>46377</v>
-      </c>
-      <c r="F28" s="11" t="n"/>
-      <c r="G28" s="11" t="n"/>
-      <c r="H28" s="9" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I28" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" s="10">
+      <c r="D28" s="7">
+        <f>IF(COUNT(D29:D35)=0,"",MIN(D29:D35))</f>
+        <v/>
+      </c>
+      <c r="E28" s="7">
+        <f>IF(COUNT(E29:E35)=0,"",MAX(E29:E35))</f>
+        <v/>
+      </c>
+      <c r="F28" s="7">
+        <f>IF(COUNT(F29:F35)=0,"",MIN(F29:F35))</f>
+        <v/>
+      </c>
+      <c r="G28" s="7">
+        <f>IF(COUNT(G29:G35)=0,"",MAX(G29:G35))</f>
+        <v/>
+      </c>
+      <c r="H28" s="5">
+        <f>IF(I28="","",IF(I28=1,"Completada",IF(I28=0,"Pendiente","En curso")))</f>
+        <v/>
+      </c>
+      <c r="I28" s="8">
+        <f>IF(COUNT(I29:I35)=0,"",AVERAGE(I29:I35))</f>
+        <v/>
+      </c>
+      <c r="J28" s="6">
         <f>IF(AND(G28&lt;&gt;"",E28&lt;&gt;""),G28-E28,"")</f>
         <v/>
       </c>
-      <c r="K28" s="9" t="n"/>
-      <c r="L28" s="9" t="n"/>
-      <c r="M28" s="9" t="n"/>
-      <c r="N28" s="9" t="n"/>
-      <c r="O28" s="9" t="n"/>
-      <c r="P28" s="9" t="n"/>
-      <c r="Q28" s="9" t="n"/>
-      <c r="R28" s="9" t="n"/>
-      <c r="S28" s="9" t="n"/>
-      <c r="T28" s="9" t="n"/>
-      <c r="U28" s="9" t="n"/>
-      <c r="V28" s="9" t="n"/>
-      <c r="W28" s="9" t="n"/>
-      <c r="X28" s="9" t="n"/>
-      <c r="Y28" s="9" t="n"/>
-      <c r="Z28" s="9" t="n"/>
-      <c r="AA28" s="9" t="n"/>
-      <c r="AB28" s="9" t="n"/>
-      <c r="AC28" s="9" t="n"/>
-      <c r="AD28" s="9" t="n"/>
-      <c r="AE28" s="9" t="n"/>
-      <c r="AF28" s="9" t="n"/>
-      <c r="AG28" s="9" t="n"/>
+      <c r="K28" s="5" t="n"/>
+      <c r="L28" s="5" t="n"/>
+      <c r="M28" s="5" t="n"/>
+      <c r="N28" s="5" t="n"/>
+      <c r="O28" s="5" t="n"/>
+      <c r="P28" s="5" t="n"/>
+      <c r="Q28" s="5" t="n"/>
+      <c r="R28" s="5" t="n"/>
+      <c r="S28" s="5" t="n"/>
+      <c r="T28" s="5" t="n"/>
+      <c r="U28" s="5" t="n"/>
+      <c r="V28" s="5" t="n"/>
+      <c r="W28" s="5" t="n"/>
+      <c r="X28" s="5" t="n"/>
+      <c r="Y28" s="5" t="n"/>
+      <c r="Z28" s="5" t="n"/>
+      <c r="AA28" s="5" t="n"/>
+      <c r="AB28" s="5" t="n"/>
+      <c r="AC28" s="5" t="n"/>
+      <c r="AD28" s="5" t="n"/>
+      <c r="AE28" s="5" t="n"/>
+      <c r="AF28" s="5" t="n"/>
+      <c r="AG28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Gestor de tareas largas (servicios `dataSync` / `mediaProcessing` con tiempo límite y reanudación por check...</t>
+          <t>`core/export`: `trip.json` + JSON Schema, GPX 1.1 con extensiones propias y de Garmin validado contra XSD,...</t>
         </is>
       </c>
       <c r="C29" s="10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>46377</v>
+        <v>46365</v>
       </c>
       <c r="E29" s="11" t="n">
-        <v>46381</v>
+        <v>46374</v>
       </c>
       <c r="F29" s="11" t="n"/>
       <c r="G29" s="11" t="n"/>
@@ -2192,22 +2204,22 @@
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Importación de `trip.json` y de GPX externo</t>
+          <t>Gestor de tareas largas (servicios `dataSync` / `mediaProcessing` con tiempo límite y reanudación por check...</t>
         </is>
       </c>
       <c r="C30" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" s="11" t="n">
-        <v>46381</v>
+        <v>46374</v>
       </c>
       <c r="E30" s="11" t="n">
-        <v>46383</v>
+        <v>46378</v>
       </c>
       <c r="F30" s="11" t="n"/>
       <c r="G30" s="11" t="n"/>
@@ -2250,22 +2262,22 @@
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>whisper.cpp con NDK (alineado a 16 KB), descarga de modelo, VAD obligatorio, confianza por segmento, `Trans...</t>
+          <t>Importación de `trip.json` y de GPX externo</t>
         </is>
       </c>
       <c r="C31" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>46383</v>
+        <v>46378</v>
       </c>
       <c r="E31" s="11" t="n">
-        <v>46390</v>
+        <v>46380</v>
       </c>
       <c r="F31" s="11" t="n"/>
       <c r="G31" s="11" t="n"/>
@@ -2308,22 +2320,22 @@
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Respaldo: base excluida del Auto Backup; `trip.json` automático al cerrar cada etapa</t>
+          <t>whisper.cpp con NDK (alineado a 16 KB), descarga de modelo, VAD obligatorio, confianza por segmento, `Trans...</t>
         </is>
       </c>
       <c r="C32" s="10" t="n">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="D32" s="11" t="n">
-        <v>46390</v>
+        <v>46380</v>
       </c>
       <c r="E32" s="11" t="n">
-        <v>46391</v>
+        <v>46387</v>
       </c>
       <c r="F32" s="11" t="n"/>
       <c r="G32" s="11" t="n"/>
@@ -2366,22 +2378,22 @@
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Nombre de ruta y detección de senderos (Nominatim, Overpass) con política de resiliencia (User-Agent, caché...</t>
+          <t>Respaldo: base excluida del Auto Backup; `trip.json` automático al cerrar cada etapa</t>
         </is>
       </c>
       <c r="C33" s="10" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D33" s="11" t="n">
-        <v>46391</v>
+        <v>46387</v>
       </c>
       <c r="E33" s="11" t="n">
-        <v>46393</v>
+        <v>46388</v>
       </c>
       <c r="F33" s="11" t="n"/>
       <c r="G33" s="11" t="n"/>
@@ -2424,22 +2436,22 @@
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>3.7</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>**(usuario)** Importar el KML en Google My Maps y abrir el HTML en la PC</t>
+          <t>Nombre de ruta y detección de senderos (Nominatim, Overpass) con política de resiliencia (User-Agent, caché...</t>
         </is>
       </c>
       <c r="C34" s="10" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D34" s="11" t="n">
-        <v>46393</v>
+        <v>46388</v>
       </c>
       <c r="E34" s="11" t="n">
-        <v>46394</v>
+        <v>46390</v>
       </c>
       <c r="F34" s="11" t="n"/>
       <c r="G34" s="11" t="n"/>
@@ -2480,148 +2492,148 @@
       <c r="AG34" s="9" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>**(usuario)** Importar el KML en Google My Maps y abrir el HTML en la PC</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D35" s="11" t="n">
+        <v>46390</v>
+      </c>
+      <c r="E35" s="11" t="n">
+        <v>46391</v>
+      </c>
+      <c r="F35" s="11" t="n"/>
+      <c r="G35" s="11" t="n"/>
+      <c r="H35" s="9" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I35" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="10">
+        <f>IF(AND(G35&lt;&gt;"",E35&lt;&gt;""),G35-E35,"")</f>
+        <v/>
+      </c>
+      <c r="K35" s="9" t="n"/>
+      <c r="L35" s="9" t="n"/>
+      <c r="M35" s="9" t="n"/>
+      <c r="N35" s="9" t="n"/>
+      <c r="O35" s="9" t="n"/>
+      <c r="P35" s="9" t="n"/>
+      <c r="Q35" s="9" t="n"/>
+      <c r="R35" s="9" t="n"/>
+      <c r="S35" s="9" t="n"/>
+      <c r="T35" s="9" t="n"/>
+      <c r="U35" s="9" t="n"/>
+      <c r="V35" s="9" t="n"/>
+      <c r="W35" s="9" t="n"/>
+      <c r="X35" s="9" t="n"/>
+      <c r="Y35" s="9" t="n"/>
+      <c r="Z35" s="9" t="n"/>
+      <c r="AA35" s="9" t="n"/>
+      <c r="AB35" s="9" t="n"/>
+      <c r="AC35" s="9" t="n"/>
+      <c r="AD35" s="9" t="n"/>
+      <c r="AE35" s="9" t="n"/>
+      <c r="AF35" s="9" t="n"/>
+      <c r="AG35" s="9" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>F4</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>Fase 4 — Enriquecimiento, video de escritorio y minivideo</t>
         </is>
       </c>
-      <c r="C35" s="6" t="n">
+      <c r="C36" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="D35" s="7">
-        <f>IF(COUNT(D36:D41)=0,"",MIN(D36:D41))</f>
-        <v/>
-      </c>
-      <c r="E35" s="7">
-        <f>IF(COUNT(E36:E41)=0,"",MAX(E36:E41))</f>
-        <v/>
-      </c>
-      <c r="F35" s="7">
-        <f>IF(COUNT(F36:F41)=0,"",MIN(F36:F41))</f>
-        <v/>
-      </c>
-      <c r="G35" s="7">
-        <f>IF(COUNT(G36:G41)=0,"",MAX(G36:G41))</f>
-        <v/>
-      </c>
-      <c r="H35" s="5">
-        <f>IF(I35="","",IF(I35=1,"Completada",IF(I35=0,"Pendiente","En curso")))</f>
-        <v/>
-      </c>
-      <c r="I35" s="8">
-        <f>IF(COUNT(I36:I41)=0,"",AVERAGE(I36:I41))</f>
-        <v/>
-      </c>
-      <c r="J35" s="6">
-        <f>IF(AND(G35&lt;&gt;"",E35&lt;&gt;""),G35-E35,"")</f>
-        <v/>
-      </c>
-      <c r="K35" s="5" t="n"/>
-      <c r="L35" s="5" t="n"/>
-      <c r="M35" s="5" t="n"/>
-      <c r="N35" s="5" t="n"/>
-      <c r="O35" s="5" t="n"/>
-      <c r="P35" s="5" t="n"/>
-      <c r="Q35" s="5" t="n"/>
-      <c r="R35" s="5" t="n"/>
-      <c r="S35" s="5" t="n"/>
-      <c r="T35" s="5" t="n"/>
-      <c r="U35" s="5" t="n"/>
-      <c r="V35" s="5" t="n"/>
-      <c r="W35" s="5" t="n"/>
-      <c r="X35" s="5" t="n"/>
-      <c r="Y35" s="5" t="n"/>
-      <c r="Z35" s="5" t="n"/>
-      <c r="AA35" s="5" t="n"/>
-      <c r="AB35" s="5" t="n"/>
-      <c r="AC35" s="5" t="n"/>
-      <c r="AD35" s="5" t="n"/>
-      <c r="AE35" s="5" t="n"/>
-      <c r="AF35" s="5" t="n"/>
-      <c r="AG35" s="5" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="9" t="inlineStr">
-        <is>
-          <t>4.1</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>Clientes Nominatim, Wikipedia (detrás de abstracción por la transición de su API), Wikidata y Overpass; cac...</t>
-        </is>
-      </c>
-      <c r="C36" s="10" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="D36" s="11" t="n">
-        <v>46394</v>
-      </c>
-      <c r="E36" s="11" t="n">
-        <v>46400</v>
-      </c>
-      <c r="F36" s="11" t="n"/>
-      <c r="G36" s="11" t="n"/>
-      <c r="H36" s="9" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I36" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J36" s="10">
+      <c r="D36" s="7">
+        <f>IF(COUNT(D37:D42)=0,"",MIN(D37:D42))</f>
+        <v/>
+      </c>
+      <c r="E36" s="7">
+        <f>IF(COUNT(E37:E42)=0,"",MAX(E37:E42))</f>
+        <v/>
+      </c>
+      <c r="F36" s="7">
+        <f>IF(COUNT(F37:F42)=0,"",MIN(F37:F42))</f>
+        <v/>
+      </c>
+      <c r="G36" s="7">
+        <f>IF(COUNT(G37:G42)=0,"",MAX(G37:G42))</f>
+        <v/>
+      </c>
+      <c r="H36" s="5">
+        <f>IF(I36="","",IF(I36=1,"Completada",IF(I36=0,"Pendiente","En curso")))</f>
+        <v/>
+      </c>
+      <c r="I36" s="8">
+        <f>IF(COUNT(I37:I42)=0,"",AVERAGE(I37:I42))</f>
+        <v/>
+      </c>
+      <c r="J36" s="6">
         <f>IF(AND(G36&lt;&gt;"",E36&lt;&gt;""),G36-E36,"")</f>
         <v/>
       </c>
-      <c r="K36" s="9" t="n"/>
-      <c r="L36" s="9" t="n"/>
-      <c r="M36" s="9" t="n"/>
-      <c r="N36" s="9" t="n"/>
-      <c r="O36" s="9" t="n"/>
-      <c r="P36" s="9" t="n"/>
-      <c r="Q36" s="9" t="n"/>
-      <c r="R36" s="9" t="n"/>
-      <c r="S36" s="9" t="n"/>
-      <c r="T36" s="9" t="n"/>
-      <c r="U36" s="9" t="n"/>
-      <c r="V36" s="9" t="n"/>
-      <c r="W36" s="9" t="n"/>
-      <c r="X36" s="9" t="n"/>
-      <c r="Y36" s="9" t="n"/>
-      <c r="Z36" s="9" t="n"/>
-      <c r="AA36" s="9" t="n"/>
-      <c r="AB36" s="9" t="n"/>
-      <c r="AC36" s="9" t="n"/>
-      <c r="AD36" s="9" t="n"/>
-      <c r="AE36" s="9" t="n"/>
-      <c r="AF36" s="9" t="n"/>
-      <c r="AG36" s="9" t="n"/>
+      <c r="K36" s="5" t="n"/>
+      <c r="L36" s="5" t="n"/>
+      <c r="M36" s="5" t="n"/>
+      <c r="N36" s="5" t="n"/>
+      <c r="O36" s="5" t="n"/>
+      <c r="P36" s="5" t="n"/>
+      <c r="Q36" s="5" t="n"/>
+      <c r="R36" s="5" t="n"/>
+      <c r="S36" s="5" t="n"/>
+      <c r="T36" s="5" t="n"/>
+      <c r="U36" s="5" t="n"/>
+      <c r="V36" s="5" t="n"/>
+      <c r="W36" s="5" t="n"/>
+      <c r="X36" s="5" t="n"/>
+      <c r="Y36" s="5" t="n"/>
+      <c r="Z36" s="5" t="n"/>
+      <c r="AA36" s="5" t="n"/>
+      <c r="AB36" s="5" t="n"/>
+      <c r="AC36" s="5" t="n"/>
+      <c r="AD36" s="5" t="n"/>
+      <c r="AE36" s="5" t="n"/>
+      <c r="AF36" s="5" t="n"/>
+      <c r="AG36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>Pantalla de lugares con aprobación/descarte y atribuciones</t>
+          <t>Clientes Nominatim, Wikipedia (detrás de abstracción por la transición de su API), Wikidata y Overpass; cac...</t>
         </is>
       </c>
       <c r="C37" s="10" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>46400</v>
+        <v>46391</v>
       </c>
       <c r="E37" s="11" t="n">
-        <v>46402</v>
+        <v>46396</v>
       </c>
       <c r="F37" s="11" t="n"/>
       <c r="G37" s="11" t="n"/>
@@ -2664,22 +2676,22 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>Reescritura opcional con modelo de lenguaje (clave del usuario en DataStore cifrado, restringida al texto f...</t>
+          <t>Pantalla de lugares con aprobación/descarte y atribuciones</t>
         </is>
       </c>
       <c r="C38" s="10" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D38" s="11" t="n">
-        <v>46402</v>
+        <v>46396</v>
       </c>
       <c r="E38" s="11" t="n">
-        <v>46403</v>
+        <v>46398</v>
       </c>
       <c r="F38" s="11" t="n"/>
       <c r="G38" s="11" t="n"/>
@@ -2722,22 +2734,22 @@
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>`core/videoplan`: planificador puro con preset "rápido 1 min" y duraciones 1/3/5/10 min, selección por favo...</t>
+          <t>Reescritura opcional con modelo de lenguaje (clave del usuario en DataStore cifrado, restringida al texto f...</t>
         </is>
       </c>
       <c r="C39" s="10" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>46403</v>
+        <v>46398</v>
       </c>
       <c r="E39" s="11" t="n">
-        <v>46406</v>
+        <v>46399</v>
       </c>
       <c r="F39" s="11" t="n"/>
       <c r="G39" s="11" t="n"/>
@@ -2780,22 +2792,22 @@
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.4</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>`desktop-renderer` (uv): CLI `plan` y `render`, mapa animado con teselas de MapTiler, Ken Burns, clips, tar...</t>
+          <t>`core/videoplan`: planificador puro con preset "rápido 1 min" y duraciones 1/3/5/10 min, selección por favo...</t>
         </is>
       </c>
       <c r="C40" s="10" t="n">
-        <v>5</v>
+        <v>1.5</v>
       </c>
       <c r="D40" s="11" t="n">
-        <v>46406</v>
+        <v>46399</v>
       </c>
       <c r="E40" s="11" t="n">
-        <v>46418</v>
+        <v>46402</v>
       </c>
       <c r="F40" s="11" t="n"/>
       <c r="G40" s="11" t="n"/>
@@ -2838,22 +2850,22 @@
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>Minivideo de 1 min en el teléfono: motor Media3 mínimo (título, fotos con Ken Burns, mapa estático por etap...</t>
+          <t>`desktop-renderer` (uv): CLI `plan` y `render`, mapa animado con teselas de MapTiler, Ken Burns, clips, tar...</t>
         </is>
       </c>
       <c r="C41" s="10" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="D41" s="11" t="n">
-        <v>46418</v>
+        <v>46402</v>
       </c>
       <c r="E41" s="11" t="n">
-        <v>46424</v>
+        <v>46413</v>
       </c>
       <c r="F41" s="11" t="n"/>
       <c r="G41" s="11" t="n"/>
@@ -2894,148 +2906,148 @@
       <c r="AG41" s="9" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Minivideo de 1 min en el teléfono: motor Media3 mínimo (título, fotos con Ken Burns, mapa estático por etap...</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D42" s="11" t="n">
+        <v>46413</v>
+      </c>
+      <c r="E42" s="11" t="n">
+        <v>46418</v>
+      </c>
+      <c r="F42" s="11" t="n"/>
+      <c r="G42" s="11" t="n"/>
+      <c r="H42" s="9" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I42" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" s="10">
+        <f>IF(AND(G42&lt;&gt;"",E42&lt;&gt;""),G42-E42,"")</f>
+        <v/>
+      </c>
+      <c r="K42" s="9" t="n"/>
+      <c r="L42" s="9" t="n"/>
+      <c r="M42" s="9" t="n"/>
+      <c r="N42" s="9" t="n"/>
+      <c r="O42" s="9" t="n"/>
+      <c r="P42" s="9" t="n"/>
+      <c r="Q42" s="9" t="n"/>
+      <c r="R42" s="9" t="n"/>
+      <c r="S42" s="9" t="n"/>
+      <c r="T42" s="9" t="n"/>
+      <c r="U42" s="9" t="n"/>
+      <c r="V42" s="9" t="n"/>
+      <c r="W42" s="9" t="n"/>
+      <c r="X42" s="9" t="n"/>
+      <c r="Y42" s="9" t="n"/>
+      <c r="Z42" s="9" t="n"/>
+      <c r="AA42" s="9" t="n"/>
+      <c r="AB42" s="9" t="n"/>
+      <c r="AC42" s="9" t="n"/>
+      <c r="AD42" s="9" t="n"/>
+      <c r="AE42" s="9" t="n"/>
+      <c r="AF42" s="9" t="n"/>
+      <c r="AG42" s="9" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>F5</t>
         </is>
       </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>Fase 5 — Video completo en el dispositivo y extras</t>
         </is>
       </c>
-      <c r="C42" s="6" t="n">
+      <c r="C43" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="D42" s="7">
-        <f>IF(COUNT(D43:D48)=0,"",MIN(D43:D48))</f>
-        <v/>
-      </c>
-      <c r="E42" s="7">
-        <f>IF(COUNT(E43:E48)=0,"",MAX(E43:E48))</f>
-        <v/>
-      </c>
-      <c r="F42" s="7">
-        <f>IF(COUNT(F43:F48)=0,"",MIN(F43:F48))</f>
-        <v/>
-      </c>
-      <c r="G42" s="7">
-        <f>IF(COUNT(G43:G48)=0,"",MAX(G43:G48))</f>
-        <v/>
-      </c>
-      <c r="H42" s="5">
-        <f>IF(I42="","",IF(I42=1,"Completada",IF(I42=0,"Pendiente","En curso")))</f>
-        <v/>
-      </c>
-      <c r="I42" s="8">
-        <f>IF(COUNT(I43:I48)=0,"",AVERAGE(I43:I48))</f>
-        <v/>
-      </c>
-      <c r="J42" s="6">
-        <f>IF(AND(G42&lt;&gt;"",E42&lt;&gt;""),G42-E42,"")</f>
-        <v/>
-      </c>
-      <c r="K42" s="5" t="n"/>
-      <c r="L42" s="5" t="n"/>
-      <c r="M42" s="5" t="n"/>
-      <c r="N42" s="5" t="n"/>
-      <c r="O42" s="5" t="n"/>
-      <c r="P42" s="5" t="n"/>
-      <c r="Q42" s="5" t="n"/>
-      <c r="R42" s="5" t="n"/>
-      <c r="S42" s="5" t="n"/>
-      <c r="T42" s="5" t="n"/>
-      <c r="U42" s="5" t="n"/>
-      <c r="V42" s="5" t="n"/>
-      <c r="W42" s="5" t="n"/>
-      <c r="X42" s="5" t="n"/>
-      <c r="Y42" s="5" t="n"/>
-      <c r="Z42" s="5" t="n"/>
-      <c r="AA42" s="5" t="n"/>
-      <c r="AB42" s="5" t="n"/>
-      <c r="AC42" s="5" t="n"/>
-      <c r="AD42" s="5" t="n"/>
-      <c r="AE42" s="5" t="n"/>
-      <c r="AF42" s="5" t="n"/>
-      <c r="AG42" s="5" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="9" t="inlineStr">
-        <is>
-          <t>5.1</t>
-        </is>
-      </c>
-      <c r="B43" s="9" t="inlineStr">
-        <is>
-          <t>Motor Media3 completo (mapa animado, clips, vista previa del plan editable) bajo el gestor de tareas largas</t>
-        </is>
-      </c>
-      <c r="C43" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="D43" s="11" t="n">
-        <v>46424</v>
-      </c>
-      <c r="E43" s="11" t="n">
-        <v>46433</v>
-      </c>
-      <c r="F43" s="11" t="n"/>
-      <c r="G43" s="11" t="n"/>
-      <c r="H43" s="9" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="I43" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J43" s="10">
+      <c r="D43" s="7">
+        <f>IF(COUNT(D44:D49)=0,"",MIN(D44:D49))</f>
+        <v/>
+      </c>
+      <c r="E43" s="7">
+        <f>IF(COUNT(E44:E49)=0,"",MAX(E44:E49))</f>
+        <v/>
+      </c>
+      <c r="F43" s="7">
+        <f>IF(COUNT(F44:F49)=0,"",MIN(F44:F49))</f>
+        <v/>
+      </c>
+      <c r="G43" s="7">
+        <f>IF(COUNT(G44:G49)=0,"",MAX(G44:G49))</f>
+        <v/>
+      </c>
+      <c r="H43" s="5">
+        <f>IF(I43="","",IF(I43=1,"Completada",IF(I43=0,"Pendiente","En curso")))</f>
+        <v/>
+      </c>
+      <c r="I43" s="8">
+        <f>IF(COUNT(I44:I49)=0,"",AVERAGE(I44:I49))</f>
+        <v/>
+      </c>
+      <c r="J43" s="6">
         <f>IF(AND(G43&lt;&gt;"",E43&lt;&gt;""),G43-E43,"")</f>
         <v/>
       </c>
-      <c r="K43" s="9" t="n"/>
-      <c r="L43" s="9" t="n"/>
-      <c r="M43" s="9" t="n"/>
-      <c r="N43" s="9" t="n"/>
-      <c r="O43" s="9" t="n"/>
-      <c r="P43" s="9" t="n"/>
-      <c r="Q43" s="9" t="n"/>
-      <c r="R43" s="9" t="n"/>
-      <c r="S43" s="9" t="n"/>
-      <c r="T43" s="9" t="n"/>
-      <c r="U43" s="9" t="n"/>
-      <c r="V43" s="9" t="n"/>
-      <c r="W43" s="9" t="n"/>
-      <c r="X43" s="9" t="n"/>
-      <c r="Y43" s="9" t="n"/>
-      <c r="Z43" s="9" t="n"/>
-      <c r="AA43" s="9" t="n"/>
-      <c r="AB43" s="9" t="n"/>
-      <c r="AC43" s="9" t="n"/>
-      <c r="AD43" s="9" t="n"/>
-      <c r="AE43" s="9" t="n"/>
-      <c r="AF43" s="9" t="n"/>
-      <c r="AG43" s="9" t="n"/>
+      <c r="K43" s="5" t="n"/>
+      <c r="L43" s="5" t="n"/>
+      <c r="M43" s="5" t="n"/>
+      <c r="N43" s="5" t="n"/>
+      <c r="O43" s="5" t="n"/>
+      <c r="P43" s="5" t="n"/>
+      <c r="Q43" s="5" t="n"/>
+      <c r="R43" s="5" t="n"/>
+      <c r="S43" s="5" t="n"/>
+      <c r="T43" s="5" t="n"/>
+      <c r="U43" s="5" t="n"/>
+      <c r="V43" s="5" t="n"/>
+      <c r="W43" s="5" t="n"/>
+      <c r="X43" s="5" t="n"/>
+      <c r="Y43" s="5" t="n"/>
+      <c r="Z43" s="5" t="n"/>
+      <c r="AA43" s="5" t="n"/>
+      <c r="AB43" s="5" t="n"/>
+      <c r="AC43" s="5" t="n"/>
+      <c r="AD43" s="5" t="n"/>
+      <c r="AE43" s="5" t="n"/>
+      <c r="AF43" s="5" t="n"/>
+      <c r="AG43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>Cámara integrada (CameraX) con EXIF GPS y nota sobre la foto</t>
+          <t>Motor Media3 completo (mapa animado, clips, vista previa del plan editable) bajo el gestor de tareas largas</t>
         </is>
       </c>
       <c r="C44" s="10" t="n">
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="D44" s="11" t="n">
-        <v>46433</v>
+        <v>46418</v>
       </c>
       <c r="E44" s="11" t="n">
-        <v>46436</v>
+        <v>46427</v>
       </c>
       <c r="F44" s="11" t="n"/>
       <c r="G44" s="11" t="n"/>
@@ -3078,22 +3090,22 @@
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>5.2</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>Widget, mosaico de Configuración rápida y accesos directos</t>
+          <t>Cámara integrada (CameraX) con EXIF GPS y nota sobre la foto</t>
         </is>
       </c>
       <c r="C45" s="10" t="n">
         <v>1.5</v>
       </c>
       <c r="D45" s="11" t="n">
-        <v>46436</v>
+        <v>46427</v>
       </c>
       <c r="E45" s="11" t="n">
-        <v>46439</v>
+        <v>46430</v>
       </c>
       <c r="F45" s="11" t="n"/>
       <c r="G45" s="11" t="n"/>
@@ -3136,22 +3148,22 @@
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>5.4</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>Mapas offline con MapLibre (descarga de región)</t>
+          <t>Widget, mosaico de Configuración rápida y accesos directos</t>
         </is>
       </c>
       <c r="C46" s="10" t="n">
         <v>1.5</v>
       </c>
       <c r="D46" s="11" t="n">
-        <v>46439</v>
+        <v>46430</v>
       </c>
       <c r="E46" s="11" t="n">
-        <v>46442</v>
+        <v>46433</v>
       </c>
       <c r="F46" s="11" t="n"/>
       <c r="G46" s="11" t="n"/>
@@ -3194,22 +3206,22 @@
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>Zonas de privacidad aplicadas al exportar</t>
+          <t>Mapas offline con MapLibre (descarga de región)</t>
         </is>
       </c>
       <c r="C47" s="10" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="D47" s="11" t="n">
-        <v>46442</v>
+        <v>46433</v>
       </c>
       <c r="E47" s="11" t="n">
-        <v>46444</v>
+        <v>46436</v>
       </c>
       <c r="F47" s="11" t="n"/>
       <c r="G47" s="11" t="n"/>
@@ -3252,27 +3264,33 @@
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>Google Fotos (Picker e importación / subida a álbum propio). DESEABLE A FUTURO (2026-10-11, usuario): requi...</t>
+          <t>Zonas de privacidad aplicadas al exportar</t>
         </is>
       </c>
       <c r="C48" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D48" s="11" t="n"/>
-      <c r="E48" s="11" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="D48" s="11" t="n">
+        <v>46436</v>
+      </c>
+      <c r="E48" s="11" t="n">
+        <v>46438</v>
+      </c>
       <c r="F48" s="11" t="n"/>
       <c r="G48" s="11" t="n"/>
       <c r="H48" s="9" t="inlineStr">
         <is>
-          <t>Deseable a futuro</t>
-        </is>
-      </c>
-      <c r="I48" s="12" t="n"/>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I48" s="12" t="n">
+        <v>0</v>
+      </c>
       <c r="J48" s="10">
         <f>IF(AND(G48&lt;&gt;"",E48&lt;&gt;""),G48-E48,"")</f>
         <v/>
@@ -3302,137 +3320,137 @@
       <c r="AG48" s="9" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>Google Fotos (Picker e importación / subida a álbum propio). DESEABLE A FUTURO (2026-10-11, usuario): requi...</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="11" t="n"/>
+      <c r="E49" s="11" t="n"/>
+      <c r="F49" s="11" t="n"/>
+      <c r="G49" s="11" t="n"/>
+      <c r="H49" s="9" t="inlineStr">
+        <is>
+          <t>Deseable a futuro</t>
+        </is>
+      </c>
+      <c r="I49" s="12" t="n"/>
+      <c r="J49" s="10">
+        <f>IF(AND(G49&lt;&gt;"",E49&lt;&gt;""),G49-E49,"")</f>
+        <v/>
+      </c>
+      <c r="K49" s="9" t="n"/>
+      <c r="L49" s="9" t="n"/>
+      <c r="M49" s="9" t="n"/>
+      <c r="N49" s="9" t="n"/>
+      <c r="O49" s="9" t="n"/>
+      <c r="P49" s="9" t="n"/>
+      <c r="Q49" s="9" t="n"/>
+      <c r="R49" s="9" t="n"/>
+      <c r="S49" s="9" t="n"/>
+      <c r="T49" s="9" t="n"/>
+      <c r="U49" s="9" t="n"/>
+      <c r="V49" s="9" t="n"/>
+      <c r="W49" s="9" t="n"/>
+      <c r="X49" s="9" t="n"/>
+      <c r="Y49" s="9" t="n"/>
+      <c r="Z49" s="9" t="n"/>
+      <c r="AA49" s="9" t="n"/>
+      <c r="AB49" s="9" t="n"/>
+      <c r="AC49" s="9" t="n"/>
+      <c r="AD49" s="9" t="n"/>
+      <c r="AE49" s="9" t="n"/>
+      <c r="AF49" s="9" t="n"/>
+      <c r="AG49" s="9" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>F6</t>
         </is>
       </c>
-      <c r="B49" s="5" t="inlineStr">
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>Fase 6 — Pulido y publicación</t>
         </is>
       </c>
-      <c r="C49" s="6" t="n">
+      <c r="C50" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="D49" s="7">
-        <f>IF(COUNT(D50:D51)=0,"",MIN(D50:D51))</f>
-        <v/>
-      </c>
-      <c r="E49" s="7">
-        <f>IF(COUNT(E50:E51)=0,"",MAX(E50:E51))</f>
-        <v/>
-      </c>
-      <c r="F49" s="7">
-        <f>IF(COUNT(F50:F51)=0,"",MIN(F50:F51))</f>
-        <v/>
-      </c>
-      <c r="G49" s="7">
-        <f>IF(COUNT(G50:G51)=0,"",MAX(G50:G51))</f>
-        <v/>
-      </c>
-      <c r="H49" s="5" t="inlineStr">
+      <c r="D50" s="7">
+        <f>IF(COUNT(D51:D52)=0,"",MIN(D51:D52))</f>
+        <v/>
+      </c>
+      <c r="E50" s="7">
+        <f>IF(COUNT(E51:E52)=0,"",MAX(E51:E52))</f>
+        <v/>
+      </c>
+      <c r="F50" s="7">
+        <f>IF(COUNT(F51:F52)=0,"",MIN(F51:F52))</f>
+        <v/>
+      </c>
+      <c r="G50" s="7">
+        <f>IF(COUNT(G51:G52)=0,"",MAX(G51:G52))</f>
+        <v/>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
         <is>
           <t>Postpuesto</t>
         </is>
       </c>
-      <c r="I49" s="8">
-        <f>IF(COUNT(I50:I51)=0,"",AVERAGE(I50:I51))</f>
-        <v/>
-      </c>
-      <c r="J49" s="6">
-        <f>IF(AND(G49&lt;&gt;"",E49&lt;&gt;""),G49-E49,"")</f>
-        <v/>
-      </c>
-      <c r="K49" s="5" t="n"/>
-      <c r="L49" s="5" t="n"/>
-      <c r="M49" s="5" t="n"/>
-      <c r="N49" s="5" t="n"/>
-      <c r="O49" s="5" t="n"/>
-      <c r="P49" s="5" t="n"/>
-      <c r="Q49" s="5" t="n"/>
-      <c r="R49" s="5" t="n"/>
-      <c r="S49" s="5" t="n"/>
-      <c r="T49" s="5" t="n"/>
-      <c r="U49" s="5" t="n"/>
-      <c r="V49" s="5" t="n"/>
-      <c r="W49" s="5" t="n"/>
-      <c r="X49" s="5" t="n"/>
-      <c r="Y49" s="5" t="n"/>
-      <c r="Z49" s="5" t="n"/>
-      <c r="AA49" s="5" t="n"/>
-      <c r="AB49" s="5" t="n"/>
-      <c r="AC49" s="5" t="n"/>
-      <c r="AD49" s="5" t="n"/>
-      <c r="AE49" s="5" t="n"/>
-      <c r="AF49" s="5" t="n"/>
-      <c r="AG49" s="5" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="9" t="inlineStr">
-        <is>
-          <t>6.1</t>
-        </is>
-      </c>
-      <c r="B50" s="9" t="inlineStr">
-        <is>
-          <t>Accesibilidad, traducciones, iconografía y onboarding final</t>
-        </is>
-      </c>
-      <c r="C50" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="D50" s="11" t="n"/>
-      <c r="E50" s="11" t="n"/>
-      <c r="F50" s="11" t="n"/>
-      <c r="G50" s="11" t="n"/>
-      <c r="H50" s="9" t="inlineStr">
-        <is>
-          <t>Postpuesto</t>
-        </is>
-      </c>
-      <c r="I50" s="12" t="n"/>
-      <c r="J50" s="10">
+      <c r="I50" s="8">
+        <f>IF(COUNT(I51:I52)=0,"",AVERAGE(I51:I52))</f>
+        <v/>
+      </c>
+      <c r="J50" s="6">
         <f>IF(AND(G50&lt;&gt;"",E50&lt;&gt;""),G50-E50,"")</f>
         <v/>
       </c>
-      <c r="K50" s="9" t="n"/>
-      <c r="L50" s="9" t="n"/>
-      <c r="M50" s="9" t="n"/>
-      <c r="N50" s="9" t="n"/>
-      <c r="O50" s="9" t="n"/>
-      <c r="P50" s="9" t="n"/>
-      <c r="Q50" s="9" t="n"/>
-      <c r="R50" s="9" t="n"/>
-      <c r="S50" s="9" t="n"/>
-      <c r="T50" s="9" t="n"/>
-      <c r="U50" s="9" t="n"/>
-      <c r="V50" s="9" t="n"/>
-      <c r="W50" s="9" t="n"/>
-      <c r="X50" s="9" t="n"/>
-      <c r="Y50" s="9" t="n"/>
-      <c r="Z50" s="9" t="n"/>
-      <c r="AA50" s="9" t="n"/>
-      <c r="AB50" s="9" t="n"/>
-      <c r="AC50" s="9" t="n"/>
-      <c r="AD50" s="9" t="n"/>
-      <c r="AE50" s="9" t="n"/>
-      <c r="AF50" s="9" t="n"/>
-      <c r="AG50" s="9" t="n"/>
+      <c r="K50" s="5" t="n"/>
+      <c r="L50" s="5" t="n"/>
+      <c r="M50" s="5" t="n"/>
+      <c r="N50" s="5" t="n"/>
+      <c r="O50" s="5" t="n"/>
+      <c r="P50" s="5" t="n"/>
+      <c r="Q50" s="5" t="n"/>
+      <c r="R50" s="5" t="n"/>
+      <c r="S50" s="5" t="n"/>
+      <c r="T50" s="5" t="n"/>
+      <c r="U50" s="5" t="n"/>
+      <c r="V50" s="5" t="n"/>
+      <c r="W50" s="5" t="n"/>
+      <c r="X50" s="5" t="n"/>
+      <c r="Y50" s="5" t="n"/>
+      <c r="Z50" s="5" t="n"/>
+      <c r="AA50" s="5" t="n"/>
+      <c r="AB50" s="5" t="n"/>
+      <c r="AC50" s="5" t="n"/>
+      <c r="AD50" s="5" t="n"/>
+      <c r="AE50" s="5" t="n"/>
+      <c r="AF50" s="5" t="n"/>
+      <c r="AG50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="B51" s="9" t="inlineStr">
         <is>
-          <t>Declaraciones de Play Console, seguridad de los datos y política de privacidad; migrar el mapa del video a...</t>
+          <t>Accesibilidad, traducciones, iconografía y onboarding final</t>
         </is>
       </c>
       <c r="C51" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D51" s="11" t="n"/>
       <c r="E51" s="11" t="n"/>
@@ -3473,16 +3491,33 @@
       <c r="AG51" s="9" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="9" t="n"/>
-      <c r="B52" s="9" t="n"/>
-      <c r="C52" s="10" t="n"/>
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>Declaraciones de Play Console, seguridad de los datos y política de privacidad; migrar el mapa del video a...</t>
+        </is>
+      </c>
+      <c r="C52" s="10" t="n">
+        <v>3</v>
+      </c>
       <c r="D52" s="11" t="n"/>
       <c r="E52" s="11" t="n"/>
       <c r="F52" s="11" t="n"/>
       <c r="G52" s="11" t="n"/>
-      <c r="H52" s="9" t="n"/>
+      <c r="H52" s="9" t="inlineStr">
+        <is>
+          <t>Postpuesto</t>
+        </is>
+      </c>
       <c r="I52" s="12" t="n"/>
-      <c r="J52" s="10" t="n"/>
+      <c r="J52" s="10">
+        <f>IF(AND(G52&lt;&gt;"",E52&lt;&gt;""),G52-E52,"")</f>
+        <v/>
+      </c>
       <c r="K52" s="9" t="n"/>
       <c r="L52" s="9" t="n"/>
       <c r="M52" s="9" t="n"/>
@@ -3509,21 +3544,14 @@
     </row>
     <row r="53">
       <c r="A53" s="9" t="n"/>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>AVANCE GLOBAL</t>
-        </is>
-      </c>
+      <c r="B53" s="9" t="n"/>
       <c r="C53" s="10" t="n"/>
       <c r="D53" s="11" t="n"/>
       <c r="E53" s="11" t="n"/>
       <c r="F53" s="11" t="n"/>
       <c r="G53" s="11" t="n"/>
       <c r="H53" s="9" t="n"/>
-      <c r="I53" s="14">
-        <f>IF(COUNT(I6,I7,I8,I9,I11,I12,I13,I14,I15,I16,I17,I19,I20,I21,I22,I23,I24,I25,I26,I28,I29,I30,I31,I32,I33,I34,I36,I37,I38,I39,I40,I41,I43,I44,I45,I46,I47,I48,I50,I51)=0,"",AVERAGE(I6,I7,I8,I9,I11,I12,I13,I14,I15,I16,I17,I19,I20,I21,I22,I23,I24,I25,I26,I28,I29,I30,I31,I32,I33,I34,I36,I37,I38,I39,I40,I41,I43,I44,I45,I46,I47,I48,I50,I51))</f>
-        <v/>
-      </c>
+      <c r="I53" s="12" t="n"/>
       <c r="J53" s="10" t="n"/>
       <c r="K53" s="9" t="n"/>
       <c r="L53" s="9" t="n"/>
@@ -3549,15 +3577,57 @@
       <c r="AF53" s="9" t="n"/>
       <c r="AG53" s="9" t="n"/>
     </row>
-    <row r="55">
-      <c r="B55" s="2" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="9" t="n"/>
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>AVANCE GLOBAL</t>
+        </is>
+      </c>
+      <c r="C54" s="10" t="n"/>
+      <c r="D54" s="11" t="n"/>
+      <c r="E54" s="11" t="n"/>
+      <c r="F54" s="11" t="n"/>
+      <c r="G54" s="11" t="n"/>
+      <c r="H54" s="9" t="n"/>
+      <c r="I54" s="14">
+        <f>IF(COUNT(I6,I7,I8,I9,I11,I12,I13,I14,I15,I16,I17,I19,I20,I21,I22,I23,I24,I25,I26,I27,I29,I30,I31,I32,I33,I34,I35,I37,I38,I39,I40,I41,I42,I44,I45,I46,I47,I48,I49,I51,I52)=0,"",AVERAGE(I6,I7,I8,I9,I11,I12,I13,I14,I15,I16,I17,I19,I20,I21,I22,I23,I24,I25,I26,I27,I29,I30,I31,I32,I33,I34,I35,I37,I38,I39,I40,I41,I42,I44,I45,I46,I47,I48,I49,I51,I52))</f>
+        <v/>
+      </c>
+      <c r="J54" s="10" t="n"/>
+      <c r="K54" s="9" t="n"/>
+      <c r="L54" s="9" t="n"/>
+      <c r="M54" s="9" t="n"/>
+      <c r="N54" s="9" t="n"/>
+      <c r="O54" s="9" t="n"/>
+      <c r="P54" s="9" t="n"/>
+      <c r="Q54" s="9" t="n"/>
+      <c r="R54" s="9" t="n"/>
+      <c r="S54" s="9" t="n"/>
+      <c r="T54" s="9" t="n"/>
+      <c r="U54" s="9" t="n"/>
+      <c r="V54" s="9" t="n"/>
+      <c r="W54" s="9" t="n"/>
+      <c r="X54" s="9" t="n"/>
+      <c r="Y54" s="9" t="n"/>
+      <c r="Z54" s="9" t="n"/>
+      <c r="AA54" s="9" t="n"/>
+      <c r="AB54" s="9" t="n"/>
+      <c r="AC54" s="9" t="n"/>
+      <c r="AD54" s="9" t="n"/>
+      <c r="AE54" s="9" t="n"/>
+      <c r="AF54" s="9" t="n"/>
+      <c r="AG54" s="9" t="n"/>
+    </row>
+    <row r="56">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>Leyenda: azul = planificado · verde = real · amarillo = semana actual. Estados Descartado / Postpuesto / Deseable a futuro no cuentan para el avance.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="K5:AG52">
+  <conditionalFormatting sqref="K5:AG53">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND($G5&lt;&gt;"",K$4&lt;=$G5,K$4+6&gt;=IF($F5&lt;&gt;"",$F5,$D5))</formula>
     </cfRule>

</xml_diff>

<commit_message>
feat(export): core/export with trip.json + schema, GPX, KML/KMZ, GeoJSON, CSV, Markdown, HTML, SRT and the ZIP package (item 3.1)
- TripExport input model; one TripWriter per format; ExportPackage
  streams the ZIP, copies media/audio through a FileSource and writes
  LEEME.txt last with the database-vs-ZIP reconciliation
- docs/trip.schema.json (JSON Schema 2020-12, schema_version 1) is the
  contract with the desktop renderer; the writer is validated against it
- GPX validated against the official 1.1 XSD (test resource)
- 19 module tests; Gantt regenerated

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014MvxPtyCrWLViJ8svf2cG9
</commit_message>
<xml_diff>
--- a/reports/gantt.xlsx
+++ b/reports/gantt.xlsx
@@ -562,7 +562,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Inicio 2026-10-11 · Fin 2027-03-12 · generado 2026-10-12 desde PLAN.md</t>
+          <t>Inicio 2026-10-11 · Fin 2027-03-12 · generado 2026-10-13 desde PLAN.md</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1611,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>`MediaScanner` + observador + barrido incremental por generación (excluyendo pendientes); lectura de hora E...</t>
+          <t>`MediaScanner` + observador + barrido por ventana de la etapa (excluyendo pendientes); lectura de hora EXIF...</t>
         </is>
       </c>
       <c r="C20" s="10" t="n">
@@ -1744,14 +1744,16 @@
         <v>46354</v>
       </c>
       <c r="F22" s="11" t="n"/>
-      <c r="G22" s="11" t="n"/>
+      <c r="G22" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H22" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I22" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" s="10">
         <f>IF(AND(G22&lt;&gt;"",E22&lt;&gt;""),G22-E22,"")</f>
@@ -2040,7 +2042,9 @@
         <v>46365</v>
       </c>
       <c r="F27" s="11" t="n"/>
-      <c r="G27" s="11" t="n"/>
+      <c r="G27" s="11" t="n">
+        <v>46307</v>
+      </c>
       <c r="H27" s="9" t="inlineStr">
         <is>
           <t>Completado</t>
@@ -2167,11 +2171,11 @@
       <c r="G29" s="11" t="n"/>
       <c r="H29" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I29" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J29" s="10">
         <f>IF(AND(G29&lt;&gt;"",E29&lt;&gt;""),G29-E29,"")</f>

</xml_diff>

<commit_message>
feat(export): resumable ExportWorker with dataSync foreground, SAF/Downloads/share destinations and export dialog (item 3.2)
- StagedExport: every entry staged under cache with a manifest checkpoint;
  a retry resumes without rewriting or duplicating; ZIP assembled last
- ExportLoader: Room → TripExport with unique ZIP paths for media/audio
- ExportWorker: unique per trip (KEEP), progress notification + setProgress,
  destinations SAF (CreateDocument), MediaStore Downloads (API 29+) and
  FileProvider share; FOREGROUND_SERVICE_DATA_SYNC + SystemForegroundService
  type merged in the manifest
- Trip detail: export action, ExportDialog with options and result
- Tests: StagedExportTest (interruption + 30-day trip), ExportLoaderTest,
  dialog Compose test; emulator E2E documented

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014MvxPtyCrWLViJ8svf2cG9
</commit_message>
<xml_diff>
--- a/reports/gantt.xlsx
+++ b/reports/gantt.xlsx
@@ -2168,7 +2168,9 @@
         <v>46374</v>
       </c>
       <c r="F29" s="11" t="n"/>
-      <c r="G29" s="11" t="n"/>
+      <c r="G29" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
           <t>Completado</t>
@@ -2229,11 +2231,11 @@
       <c r="G30" s="11" t="n"/>
       <c r="H30" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I30" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J30" s="10">
         <f>IF(AND(G30&lt;&gt;"",E30&lt;&gt;""),G30-E30,"")</f>

</xml_diff>

<commit_message>
feat(import): trip.json, package ZIP and external GPX import (item 3.3)
- core/export: TripJsonReader (lenient, schema_version checked, optional id
  regeneration) and GpxReader (SAX; trk→segment, trkseg→pause, wpt→marker,
  stats and stops recomputed, synthetic times + warning when <time> is absent)
- data: TrackingRepository.importTrip in one transaction, replace by id
- app: ImportWorker (ZIP media into Pictures/BitacoraViaje via MediaStore with
  the MediaStore id kept, audio into app files), Home import action and
  result/conflict dialog
- Tests: ImportRoundTripTest (export → import copy → same database), ImportTest
  (json/gpx round trips, timeless gpx, sample trekking gpx); emulator E2E

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014MvxPtyCrWLViJ8svf2cG9
</commit_message>
<xml_diff>
--- a/reports/gantt.xlsx
+++ b/reports/gantt.xlsx
@@ -2228,7 +2228,9 @@
         <v>46378</v>
       </c>
       <c r="F30" s="11" t="n"/>
-      <c r="G30" s="11" t="n"/>
+      <c r="G30" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H30" s="9" t="inlineStr">
         <is>
           <t>Completado</t>
@@ -2289,11 +2291,11 @@
       <c r="G31" s="11" t="n"/>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I31" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31" s="10">
         <f>IF(AND(G31&lt;&gt;"",E31&lt;&gt;""),G31-E31,"")</f>

</xml_diff>

<commit_message>
feat(backup): include-only Auto Backup rules and automatic trip.json on segment close (item 3.5); CI/setup pick up the whisper submodule and NDK
- data_extraction_rules.xml / backup_rules.xml: preferences, DataStore and
  files/backup only; the database, audio and models stay out
- BackupWorker + BackupFiles.write (atomic) enqueued by finishSegment and
  finishTrip
- CI checks out submodules and installs ndk;29.0.14206865 + cmake;4.1.2;
  tools/setup-linux.sh installs the same
- BackupRulesTest (rules parsed from resources; backup file round trip)

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014MvxPtyCrWLViJ8svf2cG9
</commit_message>
<xml_diff>
--- a/reports/gantt.xlsx
+++ b/reports/gantt.xlsx
@@ -2288,7 +2288,9 @@
         <v>46380</v>
       </c>
       <c r="F31" s="11" t="n"/>
-      <c r="G31" s="11" t="n"/>
+      <c r="G31" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
           <t>Completado</t>
@@ -2407,11 +2409,11 @@
       <c r="G33" s="11" t="n"/>
       <c r="H33" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I33" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J33" s="10">
         <f>IF(AND(G33&lt;&gt;"",E33&lt;&gt;""),G33-E33,"")</f>

</xml_diff>

<commit_message>
feat(enrichment): route and trail naming from OSM with a resilient HTTP policy (item 3.6); schema v6
- core/geo: TrailMatch (coverage of a track by a named trail, merged
  parts, 60 % threshold) and RouteNaming ("RN 40, de A a B")
- app/enrichment: OsmHttp (User-Agent, cache, per-host rate limit, backoff
  on 429/503/504), NominatimClient, OverpassClient, RouteNamer,
  EnrichRouteWorker enqueued on segment close; instances changeable in
  Settings; auto name shown in the timeline, diary and trip.json
- schema v6: segment.auto_name, camera_clock_offset FK to trip,
  voice_note.media_item_id index (+ migration test)
- Tests with recorded Nominatim/Overpass answers (MockWebServer), trail
  "Sendero Madre e Hija" matched ≥ 60 %; emulator E2E documented

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014MvxPtyCrWLViJ8svf2cG9
</commit_message>
<xml_diff>
--- a/reports/gantt.xlsx
+++ b/reports/gantt.xlsx
@@ -2406,7 +2406,9 @@
         <v>46388</v>
       </c>
       <c r="F33" s="11" t="n"/>
-      <c r="G33" s="11" t="n"/>
+      <c r="G33" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H33" s="9" t="inlineStr">
         <is>
           <t>Completado</t>
@@ -2467,11 +2469,11 @@
       <c r="G34" s="11" t="n"/>
       <c r="H34" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I34" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J34" s="10">
         <f>IF(AND(G34&lt;&gt;"",E34&lt;&gt;""),G34-E34,"")</f>

</xml_diff>

<commit_message>
docs: regenerate Gantt after closing 4.1-4.5
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014MvxPtyCrWLViJ8svf2cG9
</commit_message>
<xml_diff>
--- a/reports/gantt.xlsx
+++ b/reports/gantt.xlsx
@@ -2466,7 +2466,9 @@
         <v>46390</v>
       </c>
       <c r="F34" s="11" t="n"/>
-      <c r="G34" s="11" t="n"/>
+      <c r="G34" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H34" s="9" t="inlineStr">
         <is>
           <t>Completado</t>
@@ -2648,14 +2650,16 @@
         <v>46396</v>
       </c>
       <c r="F37" s="11" t="n"/>
-      <c r="G37" s="11" t="n"/>
+      <c r="G37" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H37" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I37" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J37" s="10">
         <f>IF(AND(G37&lt;&gt;"",E37&lt;&gt;""),G37-E37,"")</f>
@@ -2706,14 +2710,16 @@
         <v>46398</v>
       </c>
       <c r="F38" s="11" t="n"/>
-      <c r="G38" s="11" t="n"/>
+      <c r="G38" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H38" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I38" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J38" s="10">
         <f>IF(AND(G38&lt;&gt;"",E38&lt;&gt;""),G38-E38,"")</f>
@@ -2764,14 +2770,16 @@
         <v>46399</v>
       </c>
       <c r="F39" s="11" t="n"/>
-      <c r="G39" s="11" t="n"/>
+      <c r="G39" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H39" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I39" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J39" s="10">
         <f>IF(AND(G39&lt;&gt;"",E39&lt;&gt;""),G39-E39,"")</f>
@@ -2822,14 +2830,16 @@
         <v>46402</v>
       </c>
       <c r="F40" s="11" t="n"/>
-      <c r="G40" s="11" t="n"/>
+      <c r="G40" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H40" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I40" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J40" s="10">
         <f>IF(AND(G40&lt;&gt;"",E40&lt;&gt;""),G40-E40,"")</f>
@@ -2880,14 +2890,16 @@
         <v>46413</v>
       </c>
       <c r="F41" s="11" t="n"/>
-      <c r="G41" s="11" t="n"/>
+      <c r="G41" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H41" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I41" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41" s="10">
         <f>IF(AND(G41&lt;&gt;"",E41&lt;&gt;""),G41-E41,"")</f>

</xml_diff>

<commit_message>
docs: regenerate Gantt after 4.6
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014MvxPtyCrWLViJ8svf2cG9
</commit_message>
<xml_diff>
--- a/reports/gantt.xlsx
+++ b/reports/gantt.xlsx
@@ -2950,14 +2950,16 @@
         <v>46418</v>
       </c>
       <c r="F42" s="11" t="n"/>
-      <c r="G42" s="11" t="n"/>
+      <c r="G42" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H42" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I42" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J42" s="10">
         <f>IF(AND(G42&lt;&gt;"",E42&lt;&gt;""),G42-E42,"")</f>

</xml_diff>

<commit_message>
docs: regenerate Gantt after 5.1
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014MvxPtyCrWLViJ8svf2cG9
</commit_message>
<xml_diff>
--- a/reports/gantt.xlsx
+++ b/reports/gantt.xlsx
@@ -3076,14 +3076,16 @@
         <v>46427</v>
       </c>
       <c r="F44" s="11" t="n"/>
-      <c r="G44" s="11" t="n"/>
+      <c r="G44" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H44" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I44" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J44" s="10">
         <f>IF(AND(G44&lt;&gt;"",E44&lt;&gt;""),G44-E44,"")</f>

</xml_diff>

<commit_message>
docs: regenerate Gantt after 5.5
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014MvxPtyCrWLViJ8svf2cG9
</commit_message>
<xml_diff>
--- a/reports/gantt.xlsx
+++ b/reports/gantt.xlsx
@@ -3310,14 +3310,16 @@
         <v>46438</v>
       </c>
       <c r="F48" s="11" t="n"/>
-      <c r="G48" s="11" t="n"/>
+      <c r="G48" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H48" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I48" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J48" s="10">
         <f>IF(AND(G48&lt;&gt;"",E48&lt;&gt;""),G48-E48,"")</f>

</xml_diff>

<commit_message>
docs: regenerate Gantt after 5.2
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014MvxPtyCrWLViJ8svf2cG9
</commit_message>
<xml_diff>
--- a/reports/gantt.xlsx
+++ b/reports/gantt.xlsx
@@ -3136,14 +3136,16 @@
         <v>46430</v>
       </c>
       <c r="F45" s="11" t="n"/>
-      <c r="G45" s="11" t="n"/>
+      <c r="G45" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H45" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I45" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J45" s="10">
         <f>IF(AND(G45&lt;&gt;"",E45&lt;&gt;""),G45-E45,"")</f>

</xml_diff>

<commit_message>
docs: regenerate Gantt after 5.3
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014MvxPtyCrWLViJ8svf2cG9
</commit_message>
<xml_diff>
--- a/reports/gantt.xlsx
+++ b/reports/gantt.xlsx
@@ -3196,14 +3196,16 @@
         <v>46433</v>
       </c>
       <c r="F46" s="11" t="n"/>
-      <c r="G46" s="11" t="n"/>
+      <c r="G46" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H46" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I46" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J46" s="10">
         <f>IF(AND(G46&lt;&gt;"",E46&lt;&gt;""),G46-E46,"")</f>
@@ -3254,14 +3256,16 @@
         <v>46436</v>
       </c>
       <c r="F47" s="11" t="n"/>
-      <c r="G47" s="11" t="n"/>
+      <c r="G47" s="11" t="n">
+        <v>46308</v>
+      </c>
       <c r="H47" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completado</t>
         </is>
       </c>
       <c r="I47" s="12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J47" s="10">
         <f>IF(AND(G47&lt;&gt;"",E47&lt;&gt;""),G47-E47,"")</f>

</xml_diff>